<commit_message>
Update column for graph_level
</commit_message>
<xml_diff>
--- a/reports/draft.xlsx
+++ b/reports/draft.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/denimoll/Files/Programming shits/dt-report-generator/reports/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AB44E0C-442E-AC4A-A6DA-990B3FA8F9E5}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65B71812-CD14-8740-B0D2-873C43975526}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="29">
   <si>
     <t>№</t>
   </si>
@@ -114,6 +114,9 @@
   </si>
   <si>
     <t>Analysis state</t>
+  </si>
+  <si>
+    <t>Graph level</t>
   </si>
 </sst>
 </file>
@@ -309,11 +312,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1453,15 +1456,16 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Таблица1" displayName="Таблица1" ref="A1:F9999" totalsRowShown="0" headerRowDxfId="8">
-  <autoFilter ref="A1:F9999" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <tableColumns count="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Таблица1" displayName="Таблица1" ref="A1:G9999" totalsRowShown="0" headerRowDxfId="8">
+  <autoFilter ref="A1:G9999" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="№" dataDxfId="7"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Dependency"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Used version" dataDxfId="6"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Group"/>
     <tableColumn id="6" xr3:uid="{285D99C5-8A98-2543-AEE5-A809E9291686}" name="Final severity"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Last version" dataDxfId="5"/>
+    <tableColumn id="7" xr3:uid="{92289575-090A-FB4E-9832-F7FD3CB66542}" name="Graph level"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight11" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1820,11 +1824,11 @@
       <c r="D7" s="8"/>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B9" s="15" t="s">
+      <c r="B9" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="15"/>
-      <c r="D9" s="15"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1841,7 +1845,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7.5" style="2" bestFit="1" customWidth="1"/>
@@ -1849,9 +1853,10 @@
     <col min="3" max="3" width="25.6640625" style="2" customWidth="1"/>
     <col min="4" max="5" width="25.6640625" customWidth="1"/>
     <col min="6" max="6" width="25.6640625" style="2" customWidth="1"/>
+    <col min="7" max="7" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1869,6 +1874,9 @@
       </c>
       <c r="F1" s="1" t="s">
         <v>10</v>
+      </c>
+      <c r="G1" s="15" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -1915,7 +1923,7 @@
       <c r="G1" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="H1" s="16" t="s">
+      <c r="H1" s="15" t="s">
         <v>27</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Rename unlnown in info
</commit_message>
<xml_diff>
--- a/reports/draft.xlsx
+++ b/reports/draft.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/denimoll/Files/Programming shits/dt-report-generator/reports/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{127ED8AE-DE3F-FF4C-AB68-8F811F2AD211}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39128873-A332-1849-9166-7ED7C44F572B}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -98,9 +98,6 @@
     <t>Low</t>
   </si>
   <si>
-    <t>Unknown</t>
-  </si>
-  <si>
     <t>All</t>
   </si>
   <si>
@@ -117,6 +114,9 @@
   </si>
   <si>
     <t>Version</t>
+  </si>
+  <si>
+    <t>Info</t>
   </si>
 </sst>
 </file>
@@ -511,7 +511,7 @@
                   <c:v>Low</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>Unknown</c:v>
+                  <c:v>Info</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -617,7 +617,7 @@
                   <c:v>Low</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>Unknown</c:v>
+                  <c:v>Info</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1876,7 +1876,7 @@
         <v>10</v>
       </c>
       <c r="G1" s="15" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -1912,19 +1912,19 @@
         <v>13</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>14</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G1" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="H1" s="15" t="s">
         <v>25</v>
-      </c>
-      <c r="H1" s="15" t="s">
-        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -1949,7 +1949,7 @@
         <v>16</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>17</v>
@@ -2009,7 +2009,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="B6" s="2">
         <f>COUNTIF('Vulnerable dependencies'!E:E,"unknown")+C6</f>

</xml_diff>